<commit_message>
Finish refactor from local regex to GRAMMAR refs.
</commit_message>
<xml_diff>
--- a/project.xlsx
+++ b/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{936F846E-1696-2342-B2BC-5EF5BCD3CCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F0CA80-AA73-B94C-9296-302D0C2A6994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40940" yWindow="-18060" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Stats" sheetId="1" r:id="rId2"/>
     <sheet name="Commands" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -169,12 +169,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -530,7 +524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EAD65B-640B-6249-BB05-DFF22DB5B4B3}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -543,13 +537,13 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -566,9 +560,27 @@
       <c r="D2">
         <v>37</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="5">
         <f>B2/D2</f>
         <v>134.83783783783784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B3">
+        <v>5630</v>
+      </c>
+      <c r="C3">
+        <v>158</v>
+      </c>
+      <c r="D3">
+        <v>41</v>
+      </c>
+      <c r="E3" s="5">
+        <f>B3/D3</f>
+        <v>137.3170731707317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Begin new qt3 arch - processClick2 to just return the new token.
</commit_message>
<xml_diff>
--- a/project.xlsx
+++ b/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F0CA80-AA73-B94C-9296-302D0C2A6994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D02452F-A47C-894D-858C-97E0876C80E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40940" yWindow="-18060" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -524,7 +524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EAD65B-640B-6249-BB05-DFF22DB5B4B3}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -581,6 +581,24 @@
       <c r="E3" s="5">
         <f>B3/D3</f>
         <v>137.3170731707317</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B4">
+        <v>5732</v>
+      </c>
+      <c r="C4">
+        <v>156</v>
+      </c>
+      <c r="D4">
+        <v>42</v>
+      </c>
+      <c r="E4" s="5">
+        <f>B4/D4</f>
+        <v>136.47619047619048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add core dir to hold invariant method.
</commit_message>
<xml_diff>
--- a/project.xlsx
+++ b/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D02452F-A47C-894D-858C-97E0876C80E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF17911-28BC-B14A-B773-8B1AEDCF6619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40940" yWindow="-18060" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -524,7 +524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EAD65B-640B-6249-BB05-DFF22DB5B4B3}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -599,6 +599,27 @@
       <c r="E4" s="5">
         <f>B4/D4</f>
         <v>136.47619047619048</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>46088</v>
+      </c>
+      <c r="B5">
+        <v>6090</v>
+      </c>
+      <c r="C5">
+        <v>167</v>
+      </c>
+      <c r="D5">
+        <v>42</v>
+      </c>
+      <c r="E5" s="5">
+        <f>B5/D5</f>
+        <v>145</v>
+      </c>
+      <c r="F5">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aborted refactor attempt on loadGame and squareClicks.
</commit_message>
<xml_diff>
--- a/project.xlsx
+++ b/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308DFDB6-D7C4-A84E-A78C-1217286D1291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B17E49-DEA3-8947-948B-9D59C632D354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-16940" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EAD65B-640B-6249-BB05-DFF22DB5B4B3}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -680,6 +680,27 @@
       </c>
       <c r="F7">
         <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="6">
+        <v>46092</v>
+      </c>
+      <c r="B8">
+        <v>6357</v>
+      </c>
+      <c r="C8">
+        <v>179</v>
+      </c>
+      <c r="D8">
+        <v>43</v>
+      </c>
+      <c r="E8" s="4">
+        <f>B8/D8</f>
+        <v>147.83720930232559</v>
+      </c>
+      <c r="F8">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Begin to cannonize regression test files.
</commit_message>
<xml_diff>
--- a/project.xlsx
+++ b/project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adgoff/Documents/Publish/WebSites/HugoExample/paradigmsage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308DFDB6-D7C4-A84E-A78C-1217286D1291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D035DFDE-C416-AA4A-99C5-06085E4155CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49160" yWindow="-16940" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{578FBB5F-CD1D-7949-925F-19C3E59B14EC}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EAD65B-640B-6249-BB05-DFF22DB5B4B3}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="6"/>
@@ -679,6 +679,66 @@
         <v>131.86046511627907</v>
       </c>
       <c r="F7">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="6">
+        <v>46092</v>
+      </c>
+      <c r="B8">
+        <v>6357</v>
+      </c>
+      <c r="C8">
+        <v>179</v>
+      </c>
+      <c r="D8">
+        <v>43</v>
+      </c>
+      <c r="E8" s="4">
+        <f>B8/D8</f>
+        <v>147.83720930232559</v>
+      </c>
+      <c r="F8">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="6">
+        <v>46093</v>
+      </c>
+      <c r="E9" s="4" t="e">
+        <f t="shared" ref="E9:E11" si="0">B9/D9</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="6">
+        <v>46094</v>
+      </c>
+      <c r="E10" s="4" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="6">
+        <v>46095</v>
+      </c>
+      <c r="B11">
+        <v>5691</v>
+      </c>
+      <c r="C11">
+        <v>153</v>
+      </c>
+      <c r="D11">
+        <v>43</v>
+      </c>
+      <c r="E11" s="4">
+        <f t="shared" si="0"/>
+        <v>132.34883720930233</v>
+      </c>
+      <c r="F11">
         <v>70</v>
       </c>
     </row>

</xml_diff>